<commit_message>
Finalized 2002 and 2003 FISE and corrected water holding data throughout
</commit_message>
<xml_diff>
--- a/Data/2022_F013B4_CO_IRATE/2022_F013B4_CO_IRATE_SoilAnalysis.xlsx
+++ b/Data/2022_F013B4_CO_IRATE/2022_F013B4_CO_IRATE_SoilAnalysis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\mnt\Data1\USDA-ALARC\GIS\PDI project\cottondata\Data\2022_F013B4_CO_IRATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F365844D-FFDE-45F2-A450-C48471E32771}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{002ADDEE-FC1D-4B71-B9B9-00DAF0B87F3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-1665" yWindow="-28410" windowWidth="27270" windowHeight="17295" xr2:uid="{9E8A4DA9-72AD-457E-9BCB-941019648664}"/>
+    <workbookView xWindow="-1470" yWindow="-24525" windowWidth="17775" windowHeight="24285" xr2:uid="{9E8A4DA9-72AD-457E-9BCB-941019648664}"/>
   </bookViews>
   <sheets>
     <sheet name="SoilDJH" sheetId="4" r:id="rId1"/>
@@ -1255,58 +1255,58 @@
         <v>27.659604999999999</v>
       </c>
       <c r="X3">
-        <v>9.4169000000000003E-2</v>
+        <v>0.15067</v>
       </c>
       <c r="Y3">
-        <v>9.8200999999999997E-2</v>
+        <v>0.15736800000000001</v>
       </c>
       <c r="Z3">
-        <v>9.7219E-2</v>
+        <v>0.15554999999999999</v>
       </c>
       <c r="AA3">
-        <v>0.100157</v>
+        <v>0.160251</v>
       </c>
       <c r="AB3">
-        <v>0.101327</v>
+        <v>0.16212399999999999</v>
       </c>
       <c r="AC3">
-        <v>9.0319999999999998E-2</v>
+        <v>0.14451</v>
       </c>
       <c r="AD3">
-        <v>0.106292</v>
+        <v>0.170067</v>
       </c>
       <c r="AE3">
-        <v>0.11140600000000001</v>
+        <v>0.17824899999999999</v>
       </c>
       <c r="AF3">
-        <v>0.10946599999999999</v>
+        <v>0.175145</v>
       </c>
       <c r="AG3">
-        <v>0.115477</v>
+        <v>0.18476300000000001</v>
       </c>
       <c r="AH3">
-        <v>0.110306</v>
+        <v>0.175065</v>
       </c>
       <c r="AI3">
-        <v>0.108408</v>
+        <v>0.17301900000000001</v>
       </c>
       <c r="AJ3">
-        <v>0.17030300000000001</v>
+        <v>0.272484</v>
       </c>
       <c r="AK3">
-        <v>0.16500799999999999</v>
+        <v>0.264013</v>
       </c>
       <c r="AL3">
-        <v>0.16723399999999999</v>
+        <v>0.27593099999999998</v>
       </c>
       <c r="AM3">
-        <v>0.17974699999999999</v>
+        <v>0.28911599999999998</v>
       </c>
       <c r="AN3">
-        <v>0.18876799999999999</v>
+        <v>0.29674499999999998</v>
       </c>
       <c r="AO3">
-        <v>0.18942000000000001</v>
+        <v>0.30017100000000002</v>
       </c>
       <c r="AP3">
         <v>54.572538999999999</v>
@@ -1568,58 +1568,58 @@
         <v>28.122332</v>
       </c>
       <c r="X5">
-        <v>9.5558000000000004E-2</v>
+        <v>0.152893</v>
       </c>
       <c r="Y5">
-        <v>9.9210999999999994E-2</v>
+        <v>0.15840499999999999</v>
       </c>
       <c r="Z5">
-        <v>9.8443000000000003E-2</v>
+        <v>0.15750900000000001</v>
       </c>
       <c r="AA5">
-        <v>9.7154000000000004E-2</v>
+        <v>0.155446</v>
       </c>
       <c r="AB5">
-        <v>9.8496E-2</v>
+        <v>0.15759300000000001</v>
       </c>
       <c r="AC5">
-        <v>9.7036999999999998E-2</v>
+        <v>0.15526400000000001</v>
       </c>
       <c r="AD5">
-        <v>0.10852100000000001</v>
+        <v>0.17363400000000001</v>
       </c>
       <c r="AE5">
-        <v>0.114638</v>
+        <v>0.183421</v>
       </c>
       <c r="AF5">
-        <v>0.109893</v>
+        <v>0.17582900000000001</v>
       </c>
       <c r="AG5">
-        <v>0.110454</v>
+        <v>0.176727</v>
       </c>
       <c r="AH5">
-        <v>0.10728</v>
+        <v>0.170987</v>
       </c>
       <c r="AI5">
-        <v>0.10895000000000001</v>
+        <v>0.173649</v>
       </c>
       <c r="AJ5">
-        <v>0.173316</v>
+        <v>0.27730500000000002</v>
       </c>
       <c r="AK5">
-        <v>0.16918800000000001</v>
+        <v>0.27070100000000002</v>
       </c>
       <c r="AL5">
-        <v>0.17710799999999999</v>
+        <v>0.28667700000000002</v>
       </c>
       <c r="AM5">
-        <v>0.18130399999999999</v>
+        <v>0.29080699999999998</v>
       </c>
       <c r="AN5">
-        <v>0.18553900000000001</v>
+        <v>0.293408</v>
       </c>
       <c r="AO5">
-        <v>0.18888199999999999</v>
+        <v>0.29969200000000001</v>
       </c>
       <c r="AP5">
         <v>54.576089000000003</v>
@@ -1881,58 +1881,58 @@
         <v>28.076982999999998</v>
       </c>
       <c r="X7">
-        <v>9.6306000000000003E-2</v>
+        <v>0.15409</v>
       </c>
       <c r="Y7">
-        <v>0.101435</v>
+        <v>0.159882</v>
       </c>
       <c r="Z7">
-        <v>9.1023000000000007E-2</v>
+        <v>0.14563699999999999</v>
       </c>
       <c r="AA7">
-        <v>8.5796999999999998E-2</v>
+        <v>0.13727500000000001</v>
       </c>
       <c r="AB7">
-        <v>9.2430999999999999E-2</v>
+        <v>0.14788899999999999</v>
       </c>
       <c r="AC7">
-        <v>9.5896999999999996E-2</v>
+        <v>0.15343699999999999</v>
       </c>
       <c r="AD7">
-        <v>0.109556</v>
+        <v>0.175289</v>
       </c>
       <c r="AE7">
-        <v>0.114722</v>
+        <v>0.183555</v>
       </c>
       <c r="AF7">
-        <v>9.9751000000000006E-2</v>
+        <v>0.15960199999999999</v>
       </c>
       <c r="AG7">
-        <v>9.6528000000000003E-2</v>
+        <v>0.154445</v>
       </c>
       <c r="AH7">
-        <v>0.10188800000000001</v>
+        <v>0.16359499999999999</v>
       </c>
       <c r="AI7">
-        <v>0.107074</v>
+        <v>0.17086100000000001</v>
       </c>
       <c r="AJ7">
-        <v>0.17824999999999999</v>
+        <v>0.28520000000000001</v>
       </c>
       <c r="AK7">
-        <v>0.17527000000000001</v>
+        <v>0.28043200000000001</v>
       </c>
       <c r="AL7">
-        <v>0.175484</v>
+        <v>0.28498000000000001</v>
       </c>
       <c r="AM7">
-        <v>0.177262</v>
+        <v>0.28653299999999998</v>
       </c>
       <c r="AN7">
-        <v>0.17696000000000001</v>
+        <v>0.28508600000000001</v>
       </c>
       <c r="AO7">
-        <v>0.18720999999999999</v>
+        <v>0.29805700000000002</v>
       </c>
       <c r="AP7">
         <v>54.505146000000003</v>
@@ -2191,58 +2191,58 @@
         <v>28.285657</v>
       </c>
       <c r="X9">
-        <v>9.3427999999999997E-2</v>
+        <v>0.14948400000000001</v>
       </c>
       <c r="Y9">
-        <v>9.8058000000000006E-2</v>
+        <v>0.15601999999999999</v>
       </c>
       <c r="Z9">
-        <v>8.6335999999999996E-2</v>
+        <v>0.13813800000000001</v>
       </c>
       <c r="AA9">
-        <v>9.9218000000000001E-2</v>
+        <v>0.158749</v>
       </c>
       <c r="AB9">
-        <v>9.4735E-2</v>
+        <v>0.15157699999999999</v>
       </c>
       <c r="AC9">
-        <v>9.5659999999999995E-2</v>
+        <v>0.153054</v>
       </c>
       <c r="AD9">
-        <v>0.105183</v>
+        <v>0.168293</v>
       </c>
       <c r="AE9">
-        <v>0.11143599999999999</v>
+        <v>0.17829800000000001</v>
       </c>
       <c r="AF9">
-        <v>9.1638999999999998E-2</v>
+        <v>0.146623</v>
       </c>
       <c r="AG9">
-        <v>0.101358</v>
+        <v>0.16217300000000001</v>
       </c>
       <c r="AH9">
-        <v>9.9345000000000003E-2</v>
+        <v>0.16000800000000001</v>
       </c>
       <c r="AI9">
-        <v>0.10427500000000001</v>
+        <v>0.16664699999999999</v>
       </c>
       <c r="AJ9">
-        <v>0.18193899999999999</v>
+        <v>0.29110200000000003</v>
       </c>
       <c r="AK9">
-        <v>0.175903</v>
+        <v>0.28144599999999997</v>
       </c>
       <c r="AL9">
-        <v>0.166134</v>
+        <v>0.27511999999999998</v>
       </c>
       <c r="AM9">
-        <v>0.175007</v>
+        <v>0.28364299999999998</v>
       </c>
       <c r="AN9">
-        <v>0.17591200000000001</v>
+        <v>0.28250500000000001</v>
       </c>
       <c r="AO9">
-        <v>0.186835</v>
+        <v>0.29719499999999999</v>
       </c>
       <c r="AP9">
         <v>53.983783000000003</v>
@@ -2501,58 +2501,58 @@
         <v>28.094048000000001</v>
       </c>
       <c r="X11">
-        <v>9.3497999999999998E-2</v>
+        <v>0.14959700000000001</v>
       </c>
       <c r="Y11">
-        <v>9.4241000000000005E-2</v>
+        <v>0.151203</v>
       </c>
       <c r="Z11">
-        <v>9.8207000000000003E-2</v>
+        <v>0.15713099999999999</v>
       </c>
       <c r="AA11">
-        <v>9.2605999999999994E-2</v>
+        <v>0.14817</v>
       </c>
       <c r="AB11">
-        <v>9.3246999999999997E-2</v>
+        <v>0.14919499999999999</v>
       </c>
       <c r="AC11">
-        <v>0.112495</v>
+        <v>0.18001300000000001</v>
       </c>
       <c r="AD11">
-        <v>0.104044</v>
+        <v>0.16647100000000001</v>
       </c>
       <c r="AE11">
-        <v>0.10999</v>
+        <v>0.175984</v>
       </c>
       <c r="AF11">
-        <v>9.9714999999999998E-2</v>
+        <v>0.15954299999999999</v>
       </c>
       <c r="AG11">
-        <v>0.102169</v>
+        <v>0.16347</v>
       </c>
       <c r="AH11">
-        <v>9.6656000000000006E-2</v>
+        <v>0.15622</v>
       </c>
       <c r="AI11">
-        <v>0.101225</v>
+        <v>0.16197500000000001</v>
       </c>
       <c r="AJ11">
-        <v>0.18255299999999999</v>
+        <v>0.29208499999999998</v>
       </c>
       <c r="AK11">
-        <v>0.17461199999999999</v>
+        <v>0.27937899999999999</v>
       </c>
       <c r="AL11">
-        <v>0.17671000000000001</v>
+        <v>0.28589300000000001</v>
       </c>
       <c r="AM11">
-        <v>0.170572</v>
+        <v>0.27803800000000001</v>
       </c>
       <c r="AN11">
-        <v>0.17379500000000001</v>
+        <v>0.27897699999999997</v>
       </c>
       <c r="AO11">
-        <v>0.18457299999999999</v>
+        <v>0.294572</v>
       </c>
       <c r="AP11">
         <v>53.250307999999997</v>
@@ -2811,58 +2811,58 @@
         <v>26.816472999999998</v>
       </c>
       <c r="X13">
-        <v>9.3039999999999998E-2</v>
+        <v>0.148865</v>
       </c>
       <c r="Y13">
-        <v>9.1454999999999995E-2</v>
+        <v>0.14798900000000001</v>
       </c>
       <c r="Z13">
-        <v>9.5112000000000002E-2</v>
+        <v>0.15218000000000001</v>
       </c>
       <c r="AA13">
-        <v>7.775E-2</v>
+        <v>0.1244</v>
       </c>
       <c r="AB13">
-        <v>8.1681000000000004E-2</v>
+        <v>0.130689</v>
       </c>
       <c r="AC13">
-        <v>7.4685000000000001E-2</v>
+        <v>0.11948</v>
       </c>
       <c r="AD13">
-        <v>0.102631</v>
+        <v>0.16420899999999999</v>
       </c>
       <c r="AE13">
-        <v>0.106211</v>
+        <v>0.16993800000000001</v>
       </c>
       <c r="AF13">
-        <v>9.7592999999999999E-2</v>
+        <v>0.15614900000000001</v>
       </c>
       <c r="AG13">
-        <v>9.3431E-2</v>
+        <v>0.14949000000000001</v>
       </c>
       <c r="AH13">
-        <v>9.1922000000000004E-2</v>
+        <v>0.14974100000000001</v>
       </c>
       <c r="AI13">
-        <v>9.3525999999999998E-2</v>
+        <v>0.15110799999999999</v>
       </c>
       <c r="AJ13">
-        <v>0.178254</v>
+        <v>0.28520699999999999</v>
       </c>
       <c r="AK13">
-        <v>0.168045</v>
+        <v>0.268872</v>
       </c>
       <c r="AL13">
-        <v>0.17494699999999999</v>
+        <v>0.28523199999999999</v>
       </c>
       <c r="AM13">
-        <v>0.162192</v>
+        <v>0.26986300000000002</v>
       </c>
       <c r="AN13">
-        <v>0.16637199999999999</v>
+        <v>0.27143899999999999</v>
       </c>
       <c r="AO13">
-        <v>0.17808499999999999</v>
+        <v>0.28851700000000002</v>
       </c>
       <c r="AP13">
         <v>53.485719000000003</v>
@@ -3121,58 +3121,58 @@
         <v>26.496737</v>
       </c>
       <c r="X15">
-        <v>9.3604000000000007E-2</v>
+        <v>0.14976700000000001</v>
       </c>
       <c r="Y15">
-        <v>9.7444000000000003E-2</v>
+        <v>0.150223</v>
       </c>
       <c r="Z15">
-        <v>9.3201999999999993E-2</v>
+        <v>0.14912300000000001</v>
       </c>
       <c r="AA15">
-        <v>9.3008999999999994E-2</v>
+        <v>0.148814</v>
       </c>
       <c r="AB15">
-        <v>9.1941999999999996E-2</v>
+        <v>0.14710799999999999</v>
       </c>
       <c r="AC15">
-        <v>8.0283999999999994E-2</v>
+        <v>0.12844700000000001</v>
       </c>
       <c r="AD15">
-        <v>0.10112</v>
+        <v>0.16179299999999999</v>
       </c>
       <c r="AE15">
-        <v>0.103857</v>
+        <v>0.16617100000000001</v>
       </c>
       <c r="AF15">
-        <v>0.106817</v>
+        <v>0.170907</v>
       </c>
       <c r="AG15">
-        <v>0.100143</v>
+        <v>0.16022800000000001</v>
       </c>
       <c r="AH15">
-        <v>9.3933000000000003E-2</v>
+        <v>0.15249499999999999</v>
       </c>
       <c r="AI15">
-        <v>9.4219999999999998E-2</v>
+        <v>0.15178900000000001</v>
       </c>
       <c r="AJ15">
-        <v>0.17491699999999999</v>
+        <v>0.27986800000000001</v>
       </c>
       <c r="AK15">
-        <v>0.16358800000000001</v>
+        <v>0.26173999999999997</v>
       </c>
       <c r="AL15">
-        <v>0.19105900000000001</v>
+        <v>0.30294100000000002</v>
       </c>
       <c r="AM15">
-        <v>0.176478</v>
+        <v>0.28400599999999998</v>
       </c>
       <c r="AN15">
-        <v>0.16996700000000001</v>
+        <v>0.272901</v>
       </c>
       <c r="AO15">
-        <v>0.179567</v>
+        <v>0.28909200000000002</v>
       </c>
       <c r="AP15">
         <v>54.273968000000004</v>
@@ -3431,58 +3431,58 @@
         <v>27.205929999999999</v>
       </c>
       <c r="X17">
-        <v>8.9108999999999994E-2</v>
+        <v>0.14257300000000001</v>
       </c>
       <c r="Y17">
-        <v>8.3780999999999994E-2</v>
+        <v>0.13863200000000001</v>
       </c>
       <c r="Z17">
-        <v>8.5342000000000001E-2</v>
+        <v>0.136547</v>
       </c>
       <c r="AA17">
-        <v>8.2594000000000001E-2</v>
+        <v>0.13214999999999999</v>
       </c>
       <c r="AB17">
-        <v>8.2503000000000007E-2</v>
+        <v>0.13200400000000001</v>
       </c>
       <c r="AC17">
-        <v>8.4358000000000002E-2</v>
+        <v>0.13496900000000001</v>
       </c>
       <c r="AD17">
-        <v>0.10236000000000001</v>
+        <v>0.163776</v>
       </c>
       <c r="AE17">
-        <v>9.6962999999999994E-2</v>
+        <v>0.155141</v>
       </c>
       <c r="AF17">
-        <v>0.101913</v>
+        <v>0.16306000000000001</v>
       </c>
       <c r="AG17">
-        <v>8.9930999999999997E-2</v>
+        <v>0.14388899999999999</v>
       </c>
       <c r="AH17">
-        <v>9.1314999999999993E-2</v>
+        <v>0.149172</v>
       </c>
       <c r="AI17">
-        <v>9.7224000000000005E-2</v>
+        <v>0.155866</v>
       </c>
       <c r="AJ17">
-        <v>0.17036399999999999</v>
+        <v>0.27258199999999999</v>
       </c>
       <c r="AK17">
-        <v>0.15553900000000001</v>
+        <v>0.248863</v>
       </c>
       <c r="AL17">
-        <v>0.18512400000000001</v>
+        <v>0.29688199999999998</v>
       </c>
       <c r="AM17">
-        <v>0.16000800000000001</v>
+        <v>0.26663500000000001</v>
       </c>
       <c r="AN17">
-        <v>0.16237599999999999</v>
+        <v>0.266013</v>
       </c>
       <c r="AO17">
-        <v>0.180446</v>
+        <v>0.28945199999999999</v>
       </c>
       <c r="AP17">
         <v>55.206530999999998</v>
@@ -3640,58 +3640,58 @@
         <v>28.435258000000001</v>
       </c>
       <c r="X18">
-        <v>9.4134999999999996E-2</v>
+        <v>0.150616</v>
       </c>
       <c r="Y18">
-        <v>9.6184000000000006E-2</v>
+        <v>0.15582399999999999</v>
       </c>
       <c r="Z18">
-        <v>9.6444000000000002E-2</v>
+        <v>0.154311</v>
       </c>
       <c r="AA18">
-        <v>9.6241999999999994E-2</v>
+        <v>0.15398700000000001</v>
       </c>
       <c r="AB18">
-        <v>9.6820000000000003E-2</v>
+        <v>0.15491099999999999</v>
       </c>
       <c r="AC18">
-        <v>9.1628000000000001E-2</v>
+        <v>0.14660500000000001</v>
       </c>
       <c r="AD18">
-        <v>0.107297</v>
+        <v>0.17167499999999999</v>
       </c>
       <c r="AE18">
-        <v>0.111586</v>
+        <v>0.178538</v>
       </c>
       <c r="AF18">
-        <v>0.10902100000000001</v>
+        <v>0.174433</v>
       </c>
       <c r="AG18">
-        <v>0.11057400000000001</v>
+        <v>0.17691799999999999</v>
       </c>
       <c r="AH18">
-        <v>0.109195</v>
+        <v>0.17352500000000001</v>
       </c>
       <c r="AI18">
-        <v>0.109171</v>
+        <v>0.17408499999999999</v>
       </c>
       <c r="AJ18">
-        <v>0.173596</v>
+        <v>0.277754</v>
       </c>
       <c r="AK18">
-        <v>0.166209</v>
+        <v>0.265934</v>
       </c>
       <c r="AL18">
-        <v>0.17277000000000001</v>
+        <v>0.28238200000000002</v>
       </c>
       <c r="AM18">
-        <v>0.177981</v>
+        <v>0.287713</v>
       </c>
       <c r="AN18">
-        <v>0.186228</v>
+        <v>0.29487999999999998</v>
       </c>
       <c r="AO18">
-        <v>0.18990899999999999</v>
+        <v>0.30071799999999999</v>
       </c>
       <c r="AP18">
         <v>54.513967999999998</v>
@@ -3852,58 +3852,58 @@
         <v>28.903583999999999</v>
       </c>
       <c r="X19">
-        <v>9.4187999999999994E-2</v>
+        <v>0.150701</v>
       </c>
       <c r="Y19">
-        <v>9.5776E-2</v>
+        <v>0.15531600000000001</v>
       </c>
       <c r="Z19">
-        <v>9.6521999999999997E-2</v>
+        <v>0.15443599999999999</v>
       </c>
       <c r="AA19">
-        <v>9.6088000000000007E-2</v>
+        <v>0.15374199999999999</v>
       </c>
       <c r="AB19">
-        <v>9.5635999999999999E-2</v>
+        <v>0.15301699999999999</v>
       </c>
       <c r="AC19">
-        <v>9.1836000000000001E-2</v>
+        <v>0.14693800000000001</v>
       </c>
       <c r="AD19">
-        <v>0.107403</v>
+        <v>0.171845</v>
       </c>
       <c r="AE19">
-        <v>0.111096</v>
+        <v>0.177754</v>
       </c>
       <c r="AF19">
-        <v>0.108739</v>
+        <v>0.173983</v>
       </c>
       <c r="AG19">
-        <v>0.109669</v>
+        <v>0.17547099999999999</v>
       </c>
       <c r="AH19">
-        <v>0.108568</v>
+        <v>0.172654</v>
       </c>
       <c r="AI19">
-        <v>0.10939</v>
+        <v>0.174401</v>
       </c>
       <c r="AJ19">
-        <v>0.17490900000000001</v>
+        <v>0.27985399999999999</v>
       </c>
       <c r="AK19">
-        <v>0.167322</v>
+        <v>0.26771499999999998</v>
       </c>
       <c r="AL19">
-        <v>0.17715600000000001</v>
+        <v>0.287441</v>
       </c>
       <c r="AM19">
-        <v>0.178976</v>
+        <v>0.28887499999999999</v>
       </c>
       <c r="AN19">
-        <v>0.18495800000000001</v>
+        <v>0.29393599999999998</v>
       </c>
       <c r="AO19">
-        <v>0.190081</v>
+        <v>0.30096299999999998</v>
       </c>
       <c r="AP19">
         <v>54.395715000000003</v>
@@ -4061,58 +4061,58 @@
         <v>28.738118</v>
       </c>
       <c r="X20">
-        <v>9.5007999999999995E-2</v>
+        <v>0.15201400000000001</v>
       </c>
       <c r="Y20">
-        <v>9.7136E-2</v>
+        <v>0.156558</v>
       </c>
       <c r="Z20">
-        <v>9.6231999999999998E-2</v>
+        <v>0.153972</v>
       </c>
       <c r="AA20">
-        <v>9.4537999999999997E-2</v>
+        <v>0.15126000000000001</v>
       </c>
       <c r="AB20">
-        <v>9.5930000000000001E-2</v>
+        <v>0.15348899999999999</v>
       </c>
       <c r="AC20">
-        <v>9.5043000000000002E-2</v>
+        <v>0.15207200000000001</v>
       </c>
       <c r="AD20">
-        <v>0.108809</v>
+        <v>0.174095</v>
       </c>
       <c r="AE20">
-        <v>0.113806</v>
+        <v>0.18209</v>
       </c>
       <c r="AF20">
-        <v>0.108068</v>
+        <v>0.17290800000000001</v>
       </c>
       <c r="AG20">
-        <v>0.107906</v>
+        <v>0.17265</v>
       </c>
       <c r="AH20">
-        <v>0.106613</v>
+        <v>0.170096</v>
       </c>
       <c r="AI20">
-        <v>0.109322</v>
+        <v>0.17419699999999999</v>
       </c>
       <c r="AJ20">
-        <v>0.174924</v>
+        <v>0.27987899999999999</v>
       </c>
       <c r="AK20">
-        <v>0.169075</v>
+        <v>0.27051999999999998</v>
       </c>
       <c r="AL20">
-        <v>0.17660200000000001</v>
+        <v>0.28642200000000001</v>
       </c>
       <c r="AM20">
-        <v>0.17876400000000001</v>
+        <v>0.28844999999999998</v>
       </c>
       <c r="AN20">
-        <v>0.183564</v>
+        <v>0.29214200000000001</v>
       </c>
       <c r="AO20">
-        <v>0.18951399999999999</v>
+        <v>0.30039500000000002</v>
       </c>
       <c r="AP20">
         <v>54.553635999999997</v>
@@ -4273,58 +4273,58 @@
         <v>29.136979</v>
       </c>
       <c r="X21">
-        <v>9.4687999999999994E-2</v>
+        <v>0.1515</v>
       </c>
       <c r="Y21">
-        <v>9.6404000000000004E-2</v>
+        <v>0.15565399999999999</v>
       </c>
       <c r="Z21">
-        <v>9.5582E-2</v>
+        <v>0.15293200000000001</v>
       </c>
       <c r="AA21">
-        <v>9.4667000000000001E-2</v>
+        <v>0.15146699999999999</v>
       </c>
       <c r="AB21">
-        <v>9.5061999999999994E-2</v>
+        <v>0.15209900000000001</v>
       </c>
       <c r="AC21">
-        <v>9.3673000000000006E-2</v>
+        <v>0.14987800000000001</v>
       </c>
       <c r="AD21">
-        <v>0.10853</v>
+        <v>0.173648</v>
       </c>
       <c r="AE21">
-        <v>0.112717</v>
+        <v>0.18034700000000001</v>
       </c>
       <c r="AF21">
-        <v>0.107178</v>
+        <v>0.171484</v>
       </c>
       <c r="AG21">
-        <v>0.107712</v>
+        <v>0.17233999999999999</v>
       </c>
       <c r="AH21">
-        <v>0.10619199999999999</v>
+        <v>0.16953099999999999</v>
       </c>
       <c r="AI21">
-        <v>0.10929700000000001</v>
+        <v>0.174183</v>
       </c>
       <c r="AJ21">
-        <v>0.17577899999999999</v>
+        <v>0.281246</v>
       </c>
       <c r="AK21">
-        <v>0.16944699999999999</v>
+        <v>0.27111600000000002</v>
       </c>
       <c r="AL21">
-        <v>0.17871400000000001</v>
+        <v>0.28902499999999998</v>
       </c>
       <c r="AM21">
-        <v>0.17909600000000001</v>
+        <v>0.28892299999999999</v>
       </c>
       <c r="AN21">
-        <v>0.18255299999999999</v>
+        <v>0.29149700000000001</v>
       </c>
       <c r="AO21">
-        <v>0.189774</v>
+        <v>0.30071999999999999</v>
       </c>
       <c r="AP21">
         <v>54.346170000000001</v>
@@ -4482,58 +4482,58 @@
         <v>28.670347</v>
       </c>
       <c r="X22">
-        <v>9.5574000000000006E-2</v>
+        <v>0.152918</v>
       </c>
       <c r="Y22">
-        <v>9.9240999999999996E-2</v>
+        <v>0.15784999999999999</v>
       </c>
       <c r="Z22">
-        <v>8.8836999999999999E-2</v>
+        <v>0.14213999999999999</v>
       </c>
       <c r="AA22">
-        <v>8.2742999999999997E-2</v>
+        <v>0.13238900000000001</v>
       </c>
       <c r="AB22">
-        <v>8.9587E-2</v>
+        <v>0.14333899999999999</v>
       </c>
       <c r="AC22">
-        <v>9.3213000000000004E-2</v>
+        <v>0.14913999999999999</v>
       </c>
       <c r="AD22">
-        <v>0.109858</v>
+        <v>0.17577300000000001</v>
       </c>
       <c r="AE22">
-        <v>0.113902</v>
+        <v>0.18224299999999999</v>
       </c>
       <c r="AF22">
-        <v>9.8409999999999997E-2</v>
+        <v>0.15745500000000001</v>
       </c>
       <c r="AG22">
-        <v>9.4248999999999999E-2</v>
+        <v>0.15079799999999999</v>
       </c>
       <c r="AH22">
-        <v>0.101483</v>
+        <v>0.16306599999999999</v>
       </c>
       <c r="AI22">
-        <v>0.107447</v>
+        <v>0.171401</v>
       </c>
       <c r="AJ22">
-        <v>0.17977299999999999</v>
+        <v>0.28763699999999998</v>
       </c>
       <c r="AK22">
-        <v>0.17482500000000001</v>
+        <v>0.27972000000000002</v>
       </c>
       <c r="AL22">
-        <v>0.174287</v>
+        <v>0.28401100000000001</v>
       </c>
       <c r="AM22">
-        <v>0.17419999999999999</v>
+        <v>0.28368900000000002</v>
       </c>
       <c r="AN22">
-        <v>0.17546</v>
+        <v>0.28428999999999999</v>
       </c>
       <c r="AO22">
-        <v>0.18798699999999999</v>
+        <v>0.29885899999999999</v>
       </c>
       <c r="AP22">
         <v>54.341774000000001</v>
@@ -4694,58 +4694,58 @@
         <v>29.118625999999999</v>
       </c>
       <c r="X23">
-        <v>9.4880999999999993E-2</v>
+        <v>0.151809</v>
       </c>
       <c r="Y23">
-        <v>9.7922999999999996E-2</v>
+        <v>0.156334</v>
       </c>
       <c r="Z23">
-        <v>9.0508000000000005E-2</v>
+        <v>0.144812</v>
       </c>
       <c r="AA23">
-        <v>8.8382000000000002E-2</v>
+        <v>0.14141100000000001</v>
       </c>
       <c r="AB23">
-        <v>9.1583999999999999E-2</v>
+        <v>0.146535</v>
       </c>
       <c r="AC23">
-        <v>9.3049000000000007E-2</v>
+        <v>0.14887900000000001</v>
       </c>
       <c r="AD23">
-        <v>0.109122</v>
+        <v>0.174594</v>
       </c>
       <c r="AE23">
-        <v>0.112917</v>
+        <v>0.180668</v>
       </c>
       <c r="AF23">
-        <v>0.100299</v>
+        <v>0.16047900000000001</v>
       </c>
       <c r="AG23">
-        <v>0.10008499999999999</v>
+        <v>0.160136</v>
       </c>
       <c r="AH23">
-        <v>0.101953</v>
+        <v>0.16375200000000001</v>
       </c>
       <c r="AI23">
-        <v>0.107611</v>
+        <v>0.17163900000000001</v>
       </c>
       <c r="AJ23">
-        <v>0.17899799999999999</v>
+        <v>0.28639700000000001</v>
       </c>
       <c r="AK23">
-        <v>0.173905</v>
+        <v>0.278248</v>
       </c>
       <c r="AL23">
-        <v>0.177785</v>
+        <v>0.28807700000000003</v>
       </c>
       <c r="AM23">
-        <v>0.17669899999999999</v>
+        <v>0.28636899999999998</v>
       </c>
       <c r="AN23">
-        <v>0.17666499999999999</v>
+        <v>0.28556599999999999</v>
       </c>
       <c r="AO23">
-        <v>0.18858900000000001</v>
+        <v>0.29946400000000001</v>
       </c>
       <c r="AP23">
         <v>54.150903999999997</v>
@@ -4903,58 +4903,58 @@
         <v>29.060005</v>
       </c>
       <c r="X24">
-        <v>9.3352000000000004E-2</v>
+        <v>0.149363</v>
       </c>
       <c r="Y24">
-        <v>9.7302E-2</v>
+        <v>0.154861</v>
       </c>
       <c r="Z24">
-        <v>8.9194999999999997E-2</v>
+        <v>0.14271200000000001</v>
       </c>
       <c r="AA24">
-        <v>9.6032999999999993E-2</v>
+        <v>0.15365300000000001</v>
       </c>
       <c r="AB24">
-        <v>9.4315999999999997E-2</v>
+        <v>0.15090600000000001</v>
       </c>
       <c r="AC24">
-        <v>9.9675E-2</v>
+        <v>0.15948499999999999</v>
       </c>
       <c r="AD24">
-        <v>0.106431</v>
+        <v>0.17029</v>
       </c>
       <c r="AE24">
-        <v>0.111945</v>
+        <v>0.17911099999999999</v>
       </c>
       <c r="AF24">
-        <v>9.6667000000000003E-2</v>
+        <v>0.154668</v>
       </c>
       <c r="AG24">
-        <v>0.10381</v>
+        <v>0.16609599999999999</v>
       </c>
       <c r="AH24">
-        <v>9.9794999999999995E-2</v>
+        <v>0.16065499999999999</v>
       </c>
       <c r="AI24">
-        <v>0.10539800000000001</v>
+        <v>0.168187</v>
       </c>
       <c r="AJ24">
-        <v>0.18201000000000001</v>
+        <v>0.29121599999999997</v>
       </c>
       <c r="AK24">
-        <v>0.17644899999999999</v>
+        <v>0.28231800000000001</v>
       </c>
       <c r="AL24">
-        <v>0.175096</v>
+        <v>0.28486600000000001</v>
       </c>
       <c r="AM24">
-        <v>0.17736099999999999</v>
+        <v>0.286277</v>
       </c>
       <c r="AN24">
-        <v>0.17650299999999999</v>
+        <v>0.28345300000000001</v>
       </c>
       <c r="AO24">
-        <v>0.187947</v>
+        <v>0.29823499999999997</v>
       </c>
       <c r="AP24">
         <v>53.668049000000003</v>
@@ -5115,58 +5115,58 @@
         <v>29.608397</v>
       </c>
       <c r="X25">
-        <v>9.3109999999999998E-2</v>
+        <v>0.148975</v>
       </c>
       <c r="Y25">
-        <v>9.6499000000000001E-2</v>
+        <v>0.15376400000000001</v>
       </c>
       <c r="Z25">
-        <v>9.1037999999999994E-2</v>
+        <v>0.14566000000000001</v>
       </c>
       <c r="AA25">
-        <v>9.5412999999999998E-2</v>
+        <v>0.15265999999999999</v>
       </c>
       <c r="AB25">
-        <v>9.4153000000000001E-2</v>
+        <v>0.150645</v>
       </c>
       <c r="AC25">
-        <v>9.8659999999999998E-2</v>
+        <v>0.157861</v>
       </c>
       <c r="AD25">
-        <v>0.106765</v>
+        <v>0.170823</v>
       </c>
       <c r="AE25">
-        <v>0.111625</v>
+        <v>0.17860000000000001</v>
       </c>
       <c r="AF25">
-        <v>9.9454000000000001E-2</v>
+        <v>0.15912599999999999</v>
       </c>
       <c r="AG25">
-        <v>0.105378</v>
+        <v>0.168605</v>
       </c>
       <c r="AH25">
-        <v>0.10009800000000001</v>
+        <v>0.16112499999999999</v>
       </c>
       <c r="AI25">
-        <v>0.105687</v>
+        <v>0.168604</v>
       </c>
       <c r="AJ25">
-        <v>0.18113399999999999</v>
+        <v>0.28981499999999999</v>
       </c>
       <c r="AK25">
-        <v>0.17590900000000001</v>
+        <v>0.28145500000000001</v>
       </c>
       <c r="AL25">
-        <v>0.17907899999999999</v>
+        <v>0.289379</v>
       </c>
       <c r="AM25">
-        <v>0.178699</v>
+        <v>0.287912</v>
       </c>
       <c r="AN25">
-        <v>0.17701700000000001</v>
+        <v>0.28429300000000002</v>
       </c>
       <c r="AO25">
-        <v>0.18833800000000001</v>
+        <v>0.29866300000000001</v>
       </c>
       <c r="AP25">
         <v>53.493751000000003</v>
@@ -5324,58 +5324,58 @@
         <v>29.051286999999999</v>
       </c>
       <c r="X26">
-        <v>9.2713000000000004E-2</v>
+        <v>0.148341</v>
       </c>
       <c r="Y26">
-        <v>9.4361E-2</v>
+        <v>0.150696</v>
       </c>
       <c r="Z26">
-        <v>9.8201999999999998E-2</v>
+        <v>0.15712300000000001</v>
       </c>
       <c r="AA26">
-        <v>9.6724000000000004E-2</v>
+        <v>0.15475800000000001</v>
       </c>
       <c r="AB26">
-        <v>9.5883999999999997E-2</v>
+        <v>0.153415</v>
       </c>
       <c r="AC26">
-        <v>0.114859</v>
+        <v>0.18379799999999999</v>
       </c>
       <c r="AD26">
-        <v>0.104805</v>
+        <v>0.167688</v>
       </c>
       <c r="AE26">
-        <v>0.110703</v>
+        <v>0.177125</v>
       </c>
       <c r="AF26">
-        <v>0.103601</v>
+        <v>0.16576099999999999</v>
       </c>
       <c r="AG26">
-        <v>0.108568</v>
+        <v>0.173709</v>
       </c>
       <c r="AH26">
-        <v>9.7878999999999994E-2</v>
+        <v>0.15790299999999999</v>
       </c>
       <c r="AI26">
-        <v>0.10254099999999999</v>
+        <v>0.16378899999999999</v>
       </c>
       <c r="AJ26">
-        <v>0.18317800000000001</v>
+        <v>0.29308499999999998</v>
       </c>
       <c r="AK26">
-        <v>0.17616999999999999</v>
+        <v>0.28187200000000001</v>
       </c>
       <c r="AL26">
-        <v>0.18293999999999999</v>
+        <v>0.29267100000000001</v>
       </c>
       <c r="AM26">
-        <v>0.17714299999999999</v>
+        <v>0.28498299999999999</v>
       </c>
       <c r="AN26">
-        <v>0.17645</v>
+        <v>0.28161199999999997</v>
       </c>
       <c r="AO26">
-        <v>0.18612100000000001</v>
+        <v>0.29595199999999999</v>
       </c>
       <c r="AP26">
         <v>52.893155999999998</v>
@@ -5536,58 +5536,58 @@
         <v>29.702929999999999</v>
       </c>
       <c r="X27">
-        <v>9.2133999999999994E-2</v>
+        <v>0.14741399999999999</v>
       </c>
       <c r="Y27">
-        <v>9.3804999999999999E-2</v>
+        <v>0.149862</v>
       </c>
       <c r="Z27">
-        <v>9.7267000000000006E-2</v>
+        <v>0.15562799999999999</v>
       </c>
       <c r="AA27">
-        <v>9.6398999999999999E-2</v>
+        <v>0.15423899999999999</v>
       </c>
       <c r="AB27">
-        <v>9.4964999999999994E-2</v>
+        <v>0.151945</v>
       </c>
       <c r="AC27">
-        <v>0.105485</v>
+        <v>0.16879</v>
       </c>
       <c r="AD27">
-        <v>0.10505</v>
+        <v>0.16808000000000001</v>
       </c>
       <c r="AE27">
-        <v>0.110125</v>
+        <v>0.1762</v>
       </c>
       <c r="AF27">
-        <v>0.10416499999999999</v>
+        <v>0.16666500000000001</v>
       </c>
       <c r="AG27">
-        <v>0.108552</v>
+        <v>0.173683</v>
       </c>
       <c r="AH27">
-        <v>9.8154000000000005E-2</v>
+        <v>0.158358</v>
       </c>
       <c r="AI27">
-        <v>0.102497</v>
+        <v>0.16377700000000001</v>
       </c>
       <c r="AJ27">
-        <v>0.18149000000000001</v>
+        <v>0.29038399999999998</v>
       </c>
       <c r="AK27">
-        <v>0.17524799999999999</v>
+        <v>0.28039700000000001</v>
       </c>
       <c r="AL27">
-        <v>0.18348100000000001</v>
+        <v>0.29382799999999998</v>
       </c>
       <c r="AM27">
-        <v>0.17850099999999999</v>
+        <v>0.28704499999999999</v>
       </c>
       <c r="AN27">
-        <v>0.17675199999999999</v>
+        <v>0.28239300000000001</v>
       </c>
       <c r="AO27">
-        <v>0.18618999999999999</v>
+        <v>0.29611700000000002</v>
       </c>
       <c r="AP27">
         <v>52.657916</v>
@@ -5745,58 +5745,58 @@
         <v>27.783321000000001</v>
       </c>
       <c r="X28">
-        <v>9.1856999999999994E-2</v>
+        <v>0.14697099999999999</v>
       </c>
       <c r="Y28">
-        <v>9.1028999999999999E-2</v>
+        <v>0.14704900000000001</v>
       </c>
       <c r="Z28">
-        <v>9.5009999999999997E-2</v>
+        <v>0.15201600000000001</v>
       </c>
       <c r="AA28">
-        <v>8.3206000000000002E-2</v>
+        <v>0.133129</v>
       </c>
       <c r="AB28">
-        <v>8.5239999999999996E-2</v>
+        <v>0.13638500000000001</v>
       </c>
       <c r="AC28">
-        <v>8.1030000000000005E-2</v>
+        <v>0.129639</v>
       </c>
       <c r="AD28">
-        <v>0.10351</v>
+        <v>0.16561600000000001</v>
       </c>
       <c r="AE28">
-        <v>0.107071</v>
+        <v>0.17131299999999999</v>
       </c>
       <c r="AF28">
-        <v>0.101382</v>
+        <v>0.16221099999999999</v>
       </c>
       <c r="AG28">
-        <v>0.101285</v>
+        <v>0.16205600000000001</v>
       </c>
       <c r="AH28">
-        <v>9.3242000000000005E-2</v>
+        <v>0.15153800000000001</v>
       </c>
       <c r="AI28">
-        <v>9.5055000000000001E-2</v>
+        <v>0.153198</v>
       </c>
       <c r="AJ28">
-        <v>0.17965500000000001</v>
+        <v>0.28744799999999998</v>
       </c>
       <c r="AK28">
-        <v>0.17025999999999999</v>
+        <v>0.27241500000000002</v>
       </c>
       <c r="AL28">
-        <v>0.181148</v>
+        <v>0.291792</v>
       </c>
       <c r="AM28">
-        <v>0.169435</v>
+        <v>0.27736699999999997</v>
       </c>
       <c r="AN28">
-        <v>0.16938500000000001</v>
+        <v>0.27430900000000003</v>
       </c>
       <c r="AO28">
-        <v>0.17974399999999999</v>
+        <v>0.28993999999999998</v>
       </c>
       <c r="AP28">
         <v>53.102356999999998</v>
@@ -5957,58 +5957,58 @@
         <v>28.667981000000001</v>
       </c>
       <c r="X29">
-        <v>9.1108999999999996E-2</v>
+        <v>0.14577399999999999</v>
       </c>
       <c r="Y29">
-        <v>9.0940999999999994E-2</v>
+        <v>0.14632700000000001</v>
       </c>
       <c r="Z29">
-        <v>9.5513000000000001E-2</v>
+        <v>0.15282000000000001</v>
       </c>
       <c r="AA29">
-        <v>8.8803999999999994E-2</v>
+        <v>0.14208699999999999</v>
       </c>
       <c r="AB29">
-        <v>8.8964000000000001E-2</v>
+        <v>0.142342</v>
       </c>
       <c r="AC29">
-        <v>8.6316000000000004E-2</v>
+        <v>0.138102</v>
       </c>
       <c r="AD29">
-        <v>0.104002</v>
+        <v>0.166404</v>
       </c>
       <c r="AE29">
-        <v>0.107031</v>
+        <v>0.17124900000000001</v>
       </c>
       <c r="AF29">
-        <v>0.103883</v>
+        <v>0.166212</v>
       </c>
       <c r="AG29">
-        <v>0.105092</v>
+        <v>0.16814799999999999</v>
       </c>
       <c r="AH29">
-        <v>9.4533000000000006E-2</v>
+        <v>0.153388</v>
       </c>
       <c r="AI29">
-        <v>9.6515000000000004E-2</v>
+        <v>0.15523000000000001</v>
       </c>
       <c r="AJ29">
-        <v>0.17929300000000001</v>
+        <v>0.28686800000000001</v>
       </c>
       <c r="AK29">
-        <v>0.17083899999999999</v>
+        <v>0.273343</v>
       </c>
       <c r="AL29">
-        <v>0.18365000000000001</v>
+        <v>0.29461900000000002</v>
       </c>
       <c r="AM29">
-        <v>0.174401</v>
+        <v>0.28293499999999999</v>
       </c>
       <c r="AN29">
-        <v>0.17158000000000001</v>
+        <v>0.27661400000000003</v>
       </c>
       <c r="AO29">
-        <v>0.18107000000000001</v>
+        <v>0.29110900000000001</v>
       </c>
       <c r="AP29">
         <v>52.762782000000001</v>
@@ -6166,58 +6166,58 @@
         <v>27.456737</v>
       </c>
       <c r="X30">
-        <v>9.1449000000000003E-2</v>
+        <v>0.146319</v>
       </c>
       <c r="Y30">
-        <v>9.2689999999999995E-2</v>
+        <v>0.14630299999999999</v>
       </c>
       <c r="Z30">
-        <v>9.2439999999999994E-2</v>
+        <v>0.14790400000000001</v>
       </c>
       <c r="AA30">
-        <v>9.1450000000000004E-2</v>
+        <v>0.14632000000000001</v>
       </c>
       <c r="AB30">
-        <v>9.0471999999999997E-2</v>
+        <v>0.14475499999999999</v>
       </c>
       <c r="AC30">
-        <v>8.3458000000000004E-2</v>
+        <v>0.13352800000000001</v>
       </c>
       <c r="AD30">
-        <v>0.102644</v>
+        <v>0.16422999999999999</v>
       </c>
       <c r="AE30">
-        <v>0.103702</v>
+        <v>0.16592299999999999</v>
       </c>
       <c r="AF30">
-        <v>0.10664700000000001</v>
+        <v>0.17063500000000001</v>
       </c>
       <c r="AG30">
-        <v>0.104322</v>
+        <v>0.16691500000000001</v>
       </c>
       <c r="AH30">
-        <v>9.3743000000000007E-2</v>
+        <v>0.152283</v>
       </c>
       <c r="AI30">
-        <v>9.5044000000000003E-2</v>
+        <v>0.15292900000000001</v>
       </c>
       <c r="AJ30">
-        <v>0.176676</v>
+        <v>0.28268100000000002</v>
       </c>
       <c r="AK30">
-        <v>0.165239</v>
+        <v>0.26438200000000001</v>
       </c>
       <c r="AL30">
-        <v>0.18934500000000001</v>
+        <v>0.30102099999999998</v>
       </c>
       <c r="AM30">
-        <v>0.17661299999999999</v>
+        <v>0.28457700000000002</v>
       </c>
       <c r="AN30">
-        <v>0.169847</v>
+        <v>0.273281</v>
       </c>
       <c r="AO30">
-        <v>0.18006</v>
+        <v>0.28953499999999999</v>
       </c>
       <c r="AP30">
         <v>54.107157999999998</v>
@@ -6378,58 +6378,58 @@
         <v>28.176946000000001</v>
       </c>
       <c r="X31">
-        <v>9.0300000000000005E-2</v>
+        <v>0.144481</v>
       </c>
       <c r="Y31">
-        <v>9.0538999999999994E-2</v>
+        <v>0.14427599999999999</v>
       </c>
       <c r="Z31">
-        <v>9.2923000000000006E-2</v>
+        <v>0.148677</v>
       </c>
       <c r="AA31">
-        <v>9.2280000000000001E-2</v>
+        <v>0.147648</v>
       </c>
       <c r="AB31">
-        <v>9.0942999999999996E-2</v>
+        <v>0.145508</v>
       </c>
       <c r="AC31">
-        <v>8.5943000000000006E-2</v>
+        <v>0.13750499999999999</v>
       </c>
       <c r="AD31">
-        <v>0.103431</v>
+        <v>0.165489</v>
       </c>
       <c r="AE31">
-        <v>0.103522</v>
+        <v>0.16563600000000001</v>
       </c>
       <c r="AF31">
-        <v>0.10682</v>
+        <v>0.17091200000000001</v>
       </c>
       <c r="AG31">
-        <v>0.105975</v>
+        <v>0.16955999999999999</v>
       </c>
       <c r="AH31">
-        <v>9.4044000000000003E-2</v>
+        <v>0.15278700000000001</v>
       </c>
       <c r="AI31">
-        <v>9.5735000000000001E-2</v>
+        <v>0.15390899999999999</v>
       </c>
       <c r="AJ31">
-        <v>0.177039</v>
+        <v>0.28326200000000001</v>
       </c>
       <c r="AK31">
-        <v>0.16615099999999999</v>
+        <v>0.26584200000000002</v>
       </c>
       <c r="AL31">
-        <v>0.187942</v>
+        <v>0.29954900000000001</v>
       </c>
       <c r="AM31">
-        <v>0.17736099999999999</v>
+        <v>0.285831</v>
       </c>
       <c r="AN31">
-        <v>0.170209</v>
+        <v>0.27405800000000002</v>
       </c>
       <c r="AO31">
-        <v>0.18034</v>
+        <v>0.28981299999999999</v>
       </c>
       <c r="AP31">
         <v>54.010885000000002</v>
@@ -6590,58 +6590,58 @@
         <v>27.864581000000001</v>
       </c>
       <c r="X32">
-        <v>8.8401999999999994E-2</v>
+        <v>0.14144300000000001</v>
       </c>
       <c r="Y32">
-        <v>8.2988000000000006E-2</v>
+        <v>0.13763900000000001</v>
       </c>
       <c r="Z32">
-        <v>8.6651000000000006E-2</v>
+        <v>0.13864099999999999</v>
       </c>
       <c r="AA32">
-        <v>8.6269999999999999E-2</v>
+        <v>0.13803199999999999</v>
       </c>
       <c r="AB32">
-        <v>8.5647000000000001E-2</v>
+        <v>0.13703499999999999</v>
       </c>
       <c r="AC32">
-        <v>8.6031999999999997E-2</v>
+        <v>0.13764799999999999</v>
       </c>
       <c r="AD32">
-        <v>0.103284</v>
+        <v>0.16525400000000001</v>
       </c>
       <c r="AE32">
-        <v>9.7390000000000004E-2</v>
+        <v>0.15582399999999999</v>
       </c>
       <c r="AF32">
-        <v>0.10288899999999999</v>
+        <v>0.16462299999999999</v>
       </c>
       <c r="AG32">
-        <v>9.5177999999999999E-2</v>
+        <v>0.152285</v>
       </c>
       <c r="AH32">
-        <v>9.2005000000000003E-2</v>
+        <v>0.15015100000000001</v>
       </c>
       <c r="AI32">
-        <v>9.7508999999999998E-2</v>
+        <v>0.15624299999999999</v>
       </c>
       <c r="AJ32">
-        <v>0.17225299999999999</v>
+        <v>0.27560499999999999</v>
       </c>
       <c r="AK32">
-        <v>0.15714800000000001</v>
+        <v>0.25143700000000002</v>
       </c>
       <c r="AL32">
-        <v>0.18443699999999999</v>
+        <v>0.29616399999999998</v>
       </c>
       <c r="AM32">
-        <v>0.16531599999999999</v>
+        <v>0.27254800000000001</v>
       </c>
       <c r="AN32">
-        <v>0.163913</v>
+        <v>0.26764199999999999</v>
       </c>
       <c r="AO32">
-        <v>0.18081800000000001</v>
+        <v>0.289742</v>
       </c>
       <c r="AP32">
         <v>55.147103999999999</v>
@@ -6802,58 +6802,58 @@
         <v>28.277466</v>
       </c>
       <c r="X33">
-        <v>8.8215000000000002E-2</v>
+        <v>0.14114399999999999</v>
       </c>
       <c r="Y33">
-        <v>8.4246000000000001E-2</v>
+        <v>0.13819799999999999</v>
       </c>
       <c r="Z33">
-        <v>8.9426000000000005E-2</v>
+        <v>0.14308199999999999</v>
       </c>
       <c r="AA33">
-        <v>9.0327000000000005E-2</v>
+        <v>0.14452300000000001</v>
       </c>
       <c r="AB33">
-        <v>8.8893E-2</v>
+        <v>0.14222799999999999</v>
       </c>
       <c r="AC33">
-        <v>8.7831999999999993E-2</v>
+        <v>0.14052999999999999</v>
       </c>
       <c r="AD33">
-        <v>0.103764</v>
+        <v>0.166022</v>
       </c>
       <c r="AE33">
-        <v>9.8572999999999994E-2</v>
+        <v>0.157717</v>
       </c>
       <c r="AF33">
-        <v>0.104743</v>
+        <v>0.16758799999999999</v>
       </c>
       <c r="AG33">
-        <v>0.10061100000000001</v>
+        <v>0.16097700000000001</v>
       </c>
       <c r="AH33">
-        <v>9.2867000000000005E-2</v>
+        <v>0.151448</v>
       </c>
       <c r="AI33">
-        <v>9.7337000000000007E-2</v>
+        <v>0.156031</v>
       </c>
       <c r="AJ33">
-        <v>0.17385800000000001</v>
+        <v>0.278173</v>
       </c>
       <c r="AK33">
-        <v>0.160381</v>
+        <v>0.25660899999999998</v>
       </c>
       <c r="AL33">
-        <v>0.18521000000000001</v>
+        <v>0.29690100000000003</v>
       </c>
       <c r="AM33">
-        <v>0.17105200000000001</v>
+        <v>0.27923599999999998</v>
       </c>
       <c r="AN33">
-        <v>0.16567799999999999</v>
+        <v>0.26952900000000002</v>
       </c>
       <c r="AO33">
-        <v>0.18032400000000001</v>
+        <v>0.28935699999999998</v>
       </c>
       <c r="AP33">
         <v>55.184434000000003</v>
@@ -7239,58 +7239,58 @@
         <v>27.662997000000001</v>
       </c>
       <c r="X2">
-        <v>9.4175999999999996E-2</v>
+        <v>0.15068100000000001</v>
       </c>
       <c r="Y2">
-        <v>9.8212999999999995E-2</v>
+        <v>0.15737599999999999</v>
       </c>
       <c r="Z2">
-        <v>9.7237000000000004E-2</v>
+        <v>0.15558</v>
       </c>
       <c r="AA2">
-        <v>0.10016799999999999</v>
+        <v>0.16026899999999999</v>
       </c>
       <c r="AB2">
-        <v>0.101302</v>
+        <v>0.162083</v>
       </c>
       <c r="AC2">
-        <v>9.0326000000000004E-2</v>
+        <v>0.14451900000000001</v>
       </c>
       <c r="AD2">
-        <v>0.106292</v>
+        <v>0.170067</v>
       </c>
       <c r="AE2">
-        <v>0.1114</v>
+        <v>0.17824100000000001</v>
       </c>
       <c r="AF2">
-        <v>0.10947</v>
+        <v>0.175153</v>
       </c>
       <c r="AG2">
-        <v>0.115463</v>
+        <v>0.18474199999999999</v>
       </c>
       <c r="AH2">
-        <v>0.11029</v>
+        <v>0.175042</v>
       </c>
       <c r="AI2">
-        <v>0.108404</v>
+        <v>0.173012</v>
       </c>
       <c r="AJ2">
-        <v>0.17033699999999999</v>
+        <v>0.27253899999999998</v>
       </c>
       <c r="AK2">
-        <v>0.165047</v>
+        <v>0.264075</v>
       </c>
       <c r="AL2">
-        <v>0.16738</v>
+        <v>0.27609899999999998</v>
       </c>
       <c r="AM2">
-        <v>0.17979500000000001</v>
+        <v>0.28916900000000001</v>
       </c>
       <c r="AN2">
-        <v>0.18874199999999999</v>
+        <v>0.29672100000000001</v>
       </c>
       <c r="AO2">
-        <v>0.189413</v>
+        <v>0.30016399999999999</v>
       </c>
       <c r="AP2">
         <v>54.567506000000002</v>
@@ -7451,58 +7451,58 @@
         <v>28.154304</v>
       </c>
       <c r="X3">
-        <v>9.5508999999999997E-2</v>
+        <v>0.15281500000000001</v>
       </c>
       <c r="Y3">
-        <v>9.9038000000000001E-2</v>
+        <v>0.15826599999999999</v>
       </c>
       <c r="Z3">
-        <v>9.8265000000000005E-2</v>
+        <v>0.157225</v>
       </c>
       <c r="AA3">
-        <v>9.6898999999999999E-2</v>
+        <v>0.15503900000000001</v>
       </c>
       <c r="AB3">
-        <v>9.8289000000000001E-2</v>
+        <v>0.15726200000000001</v>
       </c>
       <c r="AC3">
-        <v>9.6853999999999996E-2</v>
+        <v>0.154971</v>
       </c>
       <c r="AD3">
-        <v>0.108541</v>
+        <v>0.17366599999999999</v>
       </c>
       <c r="AE3">
-        <v>0.11458599999999999</v>
+        <v>0.183338</v>
       </c>
       <c r="AF3">
-        <v>0.109776</v>
+        <v>0.17564099999999999</v>
       </c>
       <c r="AG3">
-        <v>0.11024200000000001</v>
+        <v>0.17638699999999999</v>
       </c>
       <c r="AH3">
-        <v>0.107267</v>
+        <v>0.17096900000000001</v>
       </c>
       <c r="AI3">
-        <v>0.10897800000000001</v>
+        <v>0.17369000000000001</v>
       </c>
       <c r="AJ3">
-        <v>0.17341300000000001</v>
+        <v>0.27746100000000001</v>
       </c>
       <c r="AK3">
-        <v>0.16911499999999999</v>
+        <v>0.27058500000000002</v>
       </c>
       <c r="AL3">
-        <v>0.176871</v>
+        <v>0.286435</v>
       </c>
       <c r="AM3">
-        <v>0.181008</v>
+        <v>0.290524</v>
       </c>
       <c r="AN3">
-        <v>0.18543699999999999</v>
+        <v>0.29335299999999997</v>
       </c>
       <c r="AO3">
-        <v>0.18892900000000001</v>
+        <v>0.29974099999999998</v>
       </c>
       <c r="AP3">
         <v>54.516795000000002</v>
@@ -7663,58 +7663,58 @@
         <v>28.114132999999999</v>
       </c>
       <c r="X4">
-        <v>9.6270999999999995E-2</v>
+        <v>0.154034</v>
       </c>
       <c r="Y4">
-        <v>0.101269</v>
+        <v>0.15975</v>
       </c>
       <c r="Z4">
-        <v>9.0631000000000003E-2</v>
+        <v>0.145009</v>
       </c>
       <c r="AA4">
-        <v>8.4843000000000002E-2</v>
+        <v>0.13574900000000001</v>
       </c>
       <c r="AB4">
-        <v>9.1863E-2</v>
+        <v>0.146981</v>
       </c>
       <c r="AC4">
-        <v>9.5556000000000002E-2</v>
+        <v>0.152891</v>
       </c>
       <c r="AD4">
-        <v>0.109649</v>
+        <v>0.17543800000000001</v>
       </c>
       <c r="AE4">
-        <v>0.114686</v>
+        <v>0.18349699999999999</v>
       </c>
       <c r="AF4">
-        <v>9.9446999999999994E-2</v>
+        <v>0.15911500000000001</v>
       </c>
       <c r="AG4">
-        <v>9.5665E-2</v>
+        <v>0.15306400000000001</v>
       </c>
       <c r="AH4">
-        <v>0.10180400000000001</v>
+        <v>0.16347999999999999</v>
       </c>
       <c r="AI4">
-        <v>0.107101</v>
+        <v>0.1709</v>
       </c>
       <c r="AJ4">
-        <v>0.17851</v>
+        <v>0.28561500000000001</v>
       </c>
       <c r="AK4">
-        <v>0.175285</v>
+        <v>0.28045599999999998</v>
       </c>
       <c r="AL4">
-        <v>0.17502000000000001</v>
+        <v>0.284495</v>
       </c>
       <c r="AM4">
-        <v>0.176652</v>
+        <v>0.28593499999999999</v>
       </c>
       <c r="AN4">
-        <v>0.17668500000000001</v>
+        <v>0.28489399999999998</v>
       </c>
       <c r="AO4">
-        <v>0.187253</v>
+        <v>0.29810500000000001</v>
       </c>
       <c r="AP4">
         <v>54.585327999999997</v>
@@ -7875,58 +7875,58 @@
         <v>28.288744000000001</v>
       </c>
       <c r="X5">
-        <v>9.3434000000000003E-2</v>
+        <v>0.14949399999999999</v>
       </c>
       <c r="Y5">
-        <v>9.8049999999999998E-2</v>
+        <v>0.15600900000000001</v>
       </c>
       <c r="Z5">
-        <v>8.6416000000000007E-2</v>
+        <v>0.138266</v>
       </c>
       <c r="AA5">
-        <v>9.9182000000000006E-2</v>
+        <v>0.158691</v>
       </c>
       <c r="AB5">
-        <v>9.4727000000000006E-2</v>
+        <v>0.151563</v>
       </c>
       <c r="AC5">
-        <v>9.5638000000000001E-2</v>
+        <v>0.15301999999999999</v>
       </c>
       <c r="AD5">
-        <v>0.105194</v>
+        <v>0.16831099999999999</v>
       </c>
       <c r="AE5">
-        <v>0.11143400000000001</v>
+        <v>0.17829400000000001</v>
       </c>
       <c r="AF5">
-        <v>9.1739000000000001E-2</v>
+        <v>0.146782</v>
       </c>
       <c r="AG5">
-        <v>0.101413</v>
+        <v>0.16225999999999999</v>
       </c>
       <c r="AH5">
-        <v>9.9349000000000007E-2</v>
+        <v>0.16001499999999999</v>
       </c>
       <c r="AI5">
-        <v>0.104273</v>
+        <v>0.16664399999999999</v>
       </c>
       <c r="AJ5">
-        <v>0.18190600000000001</v>
+        <v>0.291049</v>
       </c>
       <c r="AK5">
-        <v>0.17588300000000001</v>
+        <v>0.28141300000000002</v>
       </c>
       <c r="AL5">
-        <v>0.166294</v>
+        <v>0.27529900000000002</v>
       </c>
       <c r="AM5">
-        <v>0.17505200000000001</v>
+        <v>0.28369800000000001</v>
       </c>
       <c r="AN5">
-        <v>0.17591499999999999</v>
+        <v>0.28250999999999998</v>
       </c>
       <c r="AO5">
-        <v>0.18683</v>
+        <v>0.29719000000000001</v>
       </c>
       <c r="AP5">
         <v>54.157373</v>
@@ -8087,58 +8087,58 @@
         <v>28.099385999999999</v>
       </c>
       <c r="X6">
-        <v>9.3493999999999994E-2</v>
+        <v>0.14959</v>
       </c>
       <c r="Y6">
-        <v>9.4253000000000003E-2</v>
+        <v>0.15121000000000001</v>
       </c>
       <c r="Z6">
-        <v>9.8197000000000007E-2</v>
+        <v>0.157115</v>
       </c>
       <c r="AA6">
-        <v>9.2702000000000007E-2</v>
+        <v>0.14832300000000001</v>
       </c>
       <c r="AB6">
-        <v>9.3301999999999996E-2</v>
+        <v>0.149283</v>
       </c>
       <c r="AC6">
-        <v>0.112468</v>
+        <v>0.17996999999999999</v>
       </c>
       <c r="AD6">
-        <v>0.10405399999999999</v>
+        <v>0.166486</v>
       </c>
       <c r="AE6">
-        <v>0.109989</v>
+        <v>0.175982</v>
       </c>
       <c r="AF6">
-        <v>9.9768999999999997E-2</v>
+        <v>0.159631</v>
       </c>
       <c r="AG6">
-        <v>0.10231</v>
+        <v>0.16369600000000001</v>
       </c>
       <c r="AH6">
-        <v>9.6668000000000004E-2</v>
+        <v>0.15623899999999999</v>
       </c>
       <c r="AI6">
-        <v>0.101227</v>
+        <v>0.16197900000000001</v>
       </c>
       <c r="AJ6">
-        <v>0.18254000000000001</v>
+        <v>0.29206399999999999</v>
       </c>
       <c r="AK6">
-        <v>0.17461199999999999</v>
+        <v>0.27938000000000002</v>
       </c>
       <c r="AL6">
-        <v>0.176846</v>
+        <v>0.286047</v>
       </c>
       <c r="AM6">
-        <v>0.17071500000000001</v>
+        <v>0.278198</v>
       </c>
       <c r="AN6">
-        <v>0.173813</v>
+        <v>0.27899600000000002</v>
       </c>
       <c r="AO6">
-        <v>0.18457499999999999</v>
+        <v>0.294574</v>
       </c>
       <c r="AP6">
         <v>53.435665</v>
@@ -8299,58 +8299,58 @@
         <v>26.873011999999999</v>
       </c>
       <c r="X7">
-        <v>9.2954999999999996E-2</v>
+        <v>0.148728</v>
       </c>
       <c r="Y7">
-        <v>9.1411999999999993E-2</v>
+        <v>0.147924</v>
       </c>
       <c r="Z7">
-        <v>9.5076999999999995E-2</v>
+        <v>0.15212400000000001</v>
       </c>
       <c r="AA7">
-        <v>7.7996999999999997E-2</v>
+        <v>0.124795</v>
       </c>
       <c r="AB7">
-        <v>8.1835000000000005E-2</v>
+        <v>0.130936</v>
       </c>
       <c r="AC7">
-        <v>7.5013999999999997E-2</v>
+        <v>0.120007</v>
       </c>
       <c r="AD7">
-        <v>0.102696</v>
+        <v>0.16431299999999999</v>
       </c>
       <c r="AE7">
-        <v>0.106292</v>
+        <v>0.170067</v>
       </c>
       <c r="AF7">
-        <v>9.7849000000000005E-2</v>
+        <v>0.156559</v>
       </c>
       <c r="AG7">
-        <v>9.4022999999999995E-2</v>
+        <v>0.15043699999999999</v>
       </c>
       <c r="AH7">
-        <v>9.1994000000000006E-2</v>
+        <v>0.149836</v>
       </c>
       <c r="AI7">
-        <v>9.3608999999999998E-2</v>
+        <v>0.15121999999999999</v>
       </c>
       <c r="AJ7">
-        <v>0.17840800000000001</v>
+        <v>0.28545399999999999</v>
       </c>
       <c r="AK7">
-        <v>0.16823199999999999</v>
+        <v>0.26917200000000002</v>
       </c>
       <c r="AL7">
-        <v>0.17543800000000001</v>
+        <v>0.28574300000000002</v>
       </c>
       <c r="AM7">
-        <v>0.16266600000000001</v>
+        <v>0.27033600000000002</v>
       </c>
       <c r="AN7">
-        <v>0.16656699999999999</v>
+        <v>0.27161800000000003</v>
       </c>
       <c r="AO7">
-        <v>0.17818400000000001</v>
+        <v>0.288601</v>
       </c>
       <c r="AP7">
         <v>53.625788</v>
@@ -8511,58 +8511,58 @@
         <v>26.536155999999998</v>
       </c>
       <c r="X8">
-        <v>9.3493999999999994E-2</v>
+        <v>0.149591</v>
       </c>
       <c r="Y8">
-        <v>9.7169000000000005E-2</v>
+        <v>0.14998900000000001</v>
       </c>
       <c r="Z8">
-        <v>9.3118999999999993E-2</v>
+        <v>0.14899100000000001</v>
       </c>
       <c r="AA8">
-        <v>9.2953999999999995E-2</v>
+        <v>0.148726</v>
       </c>
       <c r="AB8">
-        <v>9.1873999999999997E-2</v>
+        <v>0.14699899999999999</v>
       </c>
       <c r="AC8">
-        <v>8.0523999999999998E-2</v>
+        <v>0.128832</v>
       </c>
       <c r="AD8">
-        <v>0.101187</v>
+        <v>0.16189999999999999</v>
       </c>
       <c r="AE8">
-        <v>0.103778</v>
+        <v>0.166044</v>
       </c>
       <c r="AF8">
-        <v>0.10679</v>
+        <v>0.17086499999999999</v>
       </c>
       <c r="AG8">
-        <v>0.100287</v>
+        <v>0.16045899999999999</v>
       </c>
       <c r="AH8">
-        <v>9.3909999999999993E-2</v>
+        <v>0.15246899999999999</v>
       </c>
       <c r="AI8">
-        <v>9.4283000000000006E-2</v>
+        <v>0.15187500000000001</v>
       </c>
       <c r="AJ8">
-        <v>0.17494299999999999</v>
+        <v>0.27990900000000002</v>
       </c>
       <c r="AK8">
-        <v>0.16356799999999999</v>
+        <v>0.26170900000000002</v>
       </c>
       <c r="AL8">
-        <v>0.19092799999999999</v>
+        <v>0.30280299999999999</v>
       </c>
       <c r="AM8">
-        <v>0.17641899999999999</v>
+        <v>0.283972</v>
       </c>
       <c r="AN8">
-        <v>0.169901</v>
+        <v>0.27285300000000001</v>
       </c>
       <c r="AO8">
-        <v>0.17960100000000001</v>
+        <v>0.28911599999999998</v>
       </c>
       <c r="AP8">
         <v>54.350262999999998</v>
@@ -8723,58 +8723,58 @@
         <v>27.210478999999999</v>
       </c>
       <c r="X9">
-        <v>8.9116000000000001E-2</v>
+        <v>0.14258399999999999</v>
       </c>
       <c r="Y9">
-        <v>8.3811999999999998E-2</v>
+        <v>0.13866000000000001</v>
       </c>
       <c r="Z9">
-        <v>8.5404999999999995E-2</v>
+        <v>0.13664699999999999</v>
       </c>
       <c r="AA9">
-        <v>8.2708000000000004E-2</v>
+        <v>0.13233300000000001</v>
       </c>
       <c r="AB9">
-        <v>8.2600000000000007E-2</v>
+        <v>0.13216</v>
       </c>
       <c r="AC9">
-        <v>8.4409999999999999E-2</v>
+        <v>0.13505200000000001</v>
       </c>
       <c r="AD9">
-        <v>0.102378</v>
+        <v>0.16380500000000001</v>
       </c>
       <c r="AE9">
-        <v>9.6990999999999994E-2</v>
+        <v>0.15518599999999999</v>
       </c>
       <c r="AF9">
-        <v>0.10195</v>
+        <v>0.16312099999999999</v>
       </c>
       <c r="AG9">
-        <v>9.0087E-2</v>
+        <v>0.14413899999999999</v>
       </c>
       <c r="AH9">
-        <v>9.1335E-2</v>
+        <v>0.149204</v>
       </c>
       <c r="AI9">
-        <v>9.7226000000000007E-2</v>
+        <v>0.15586900000000001</v>
       </c>
       <c r="AJ9">
-        <v>0.17041899999999999</v>
+        <v>0.27267000000000002</v>
       </c>
       <c r="AK9">
-        <v>0.15560399999999999</v>
+        <v>0.24896699999999999</v>
       </c>
       <c r="AL9">
-        <v>0.18510399999999999</v>
+        <v>0.29686099999999999</v>
       </c>
       <c r="AM9">
-        <v>0.16017400000000001</v>
+        <v>0.266822</v>
       </c>
       <c r="AN9">
-        <v>0.162415</v>
+        <v>0.26605099999999998</v>
       </c>
       <c r="AO9">
-        <v>0.180446</v>
+        <v>0.28945300000000002</v>
       </c>
       <c r="AP9">
         <v>55.271386999999997</v>
@@ -8935,58 +8935,58 @@
         <v>28.667581999999999</v>
       </c>
       <c r="X10">
-        <v>9.4161999999999996E-2</v>
+        <v>0.15065899999999999</v>
       </c>
       <c r="Y10">
-        <v>9.5998E-2</v>
+        <v>0.15558</v>
       </c>
       <c r="Z10">
-        <v>9.6491999999999994E-2</v>
+        <v>0.154387</v>
       </c>
       <c r="AA10">
-        <v>9.6210000000000004E-2</v>
+        <v>0.15393499999999999</v>
       </c>
       <c r="AB10">
-        <v>9.6269999999999994E-2</v>
+        <v>0.154032</v>
       </c>
       <c r="AC10">
-        <v>9.1717000000000007E-2</v>
+        <v>0.14674699999999999</v>
       </c>
       <c r="AD10">
-        <v>0.107337</v>
+        <v>0.171739</v>
       </c>
       <c r="AE10">
-        <v>0.111328</v>
+        <v>0.178124</v>
       </c>
       <c r="AF10">
-        <v>0.108879</v>
+        <v>0.174207</v>
       </c>
       <c r="AG10">
-        <v>0.11017100000000001</v>
+        <v>0.17627399999999999</v>
       </c>
       <c r="AH10">
-        <v>0.108887</v>
+        <v>0.173098</v>
       </c>
       <c r="AI10">
-        <v>0.109274</v>
+        <v>0.174234</v>
       </c>
       <c r="AJ10">
-        <v>0.17422599999999999</v>
+        <v>0.27876200000000001</v>
       </c>
       <c r="AK10">
-        <v>0.16676199999999999</v>
+        <v>0.26682</v>
       </c>
       <c r="AL10">
-        <v>0.17493500000000001</v>
+        <v>0.28487899999999999</v>
       </c>
       <c r="AM10">
-        <v>0.178508</v>
+        <v>0.28832099999999999</v>
       </c>
       <c r="AN10">
-        <v>0.185608</v>
+        <v>0.29441899999999999</v>
       </c>
       <c r="AO10">
-        <v>0.18999199999999999</v>
+        <v>0.30083799999999999</v>
       </c>
       <c r="AP10">
         <v>54.452618999999999</v>
@@ -9147,58 +9147,58 @@
         <v>28.937194000000002</v>
       </c>
       <c r="X11">
-        <v>9.4849000000000003E-2</v>
+        <v>0.15175900000000001</v>
       </c>
       <c r="Y11">
-        <v>9.6782000000000007E-2</v>
+        <v>0.156112</v>
       </c>
       <c r="Z11">
-        <v>9.5929E-2</v>
+        <v>0.15348600000000001</v>
       </c>
       <c r="AA11">
-        <v>9.4635999999999998E-2</v>
+        <v>0.151418</v>
       </c>
       <c r="AB11">
-        <v>9.5519000000000007E-2</v>
+        <v>0.15283099999999999</v>
       </c>
       <c r="AC11">
-        <v>9.4371999999999998E-2</v>
+        <v>0.15099799999999999</v>
       </c>
       <c r="AD11">
-        <v>0.10866099999999999</v>
+        <v>0.17385800000000001</v>
       </c>
       <c r="AE11">
-        <v>0.11325300000000001</v>
+        <v>0.181205</v>
       </c>
       <c r="AF11">
-        <v>0.107636</v>
+        <v>0.17221800000000001</v>
       </c>
       <c r="AG11">
-        <v>0.10784000000000001</v>
+        <v>0.172544</v>
       </c>
       <c r="AH11">
-        <v>0.106405</v>
+        <v>0.169818</v>
       </c>
       <c r="AI11">
-        <v>0.109305</v>
+        <v>0.17418400000000001</v>
       </c>
       <c r="AJ11">
-        <v>0.175341</v>
+        <v>0.28054499999999999</v>
       </c>
       <c r="AK11">
-        <v>0.169265</v>
+        <v>0.27082400000000001</v>
       </c>
       <c r="AL11">
-        <v>0.17768400000000001</v>
+        <v>0.28775099999999998</v>
       </c>
       <c r="AM11">
-        <v>0.17896400000000001</v>
+        <v>0.28871999999999998</v>
       </c>
       <c r="AN11">
-        <v>0.18307200000000001</v>
+        <v>0.29182900000000001</v>
       </c>
       <c r="AO11">
-        <v>0.189641</v>
+        <v>0.30055500000000002</v>
       </c>
       <c r="AP11">
         <v>54.445467999999998</v>
@@ -9359,58 +9359,58 @@
         <v>28.903115</v>
       </c>
       <c r="X12">
-        <v>9.5213999999999993E-2</v>
+        <v>0.15234200000000001</v>
       </c>
       <c r="Y12">
-        <v>9.8559999999999995E-2</v>
+        <v>0.15706200000000001</v>
       </c>
       <c r="Z12">
-        <v>8.9703000000000005E-2</v>
+        <v>0.14352500000000001</v>
       </c>
       <c r="AA12">
-        <v>8.5614999999999997E-2</v>
+        <v>0.13698399999999999</v>
       </c>
       <c r="AB12">
-        <v>9.0603000000000003E-2</v>
+        <v>0.14496500000000001</v>
       </c>
       <c r="AC12">
-        <v>9.3126E-2</v>
+        <v>0.14900099999999999</v>
       </c>
       <c r="AD12">
-        <v>0.109472</v>
+        <v>0.17515600000000001</v>
       </c>
       <c r="AE12">
-        <v>0.113381</v>
+        <v>0.18140999999999999</v>
       </c>
       <c r="AF12">
-        <v>9.9384E-2</v>
+        <v>0.15901499999999999</v>
       </c>
       <c r="AG12">
-        <v>9.7221000000000002E-2</v>
+        <v>0.155554</v>
       </c>
       <c r="AH12">
-        <v>0.10172200000000001</v>
+        <v>0.16341700000000001</v>
       </c>
       <c r="AI12">
-        <v>0.107525</v>
+        <v>0.171515</v>
       </c>
       <c r="AJ12">
-        <v>0.17937700000000001</v>
+        <v>0.28700300000000001</v>
       </c>
       <c r="AK12">
-        <v>0.17435300000000001</v>
+        <v>0.27896500000000002</v>
       </c>
       <c r="AL12">
-        <v>0.17608499999999999</v>
+        <v>0.28610099999999999</v>
       </c>
       <c r="AM12">
-        <v>0.175486</v>
+        <v>0.28506799999999999</v>
       </c>
       <c r="AN12">
-        <v>0.17608299999999999</v>
+        <v>0.28494999999999998</v>
       </c>
       <c r="AO12">
-        <v>0.18829499999999999</v>
+        <v>0.29916900000000002</v>
       </c>
       <c r="AP12">
         <v>54.238413000000001</v>
@@ -9571,58 +9571,58 @@
         <v>29.332992000000001</v>
       </c>
       <c r="X13">
-        <v>9.3225000000000002E-2</v>
+        <v>0.14915999999999999</v>
       </c>
       <c r="Y13">
-        <v>9.6895999999999996E-2</v>
+        <v>0.154307</v>
       </c>
       <c r="Z13">
-        <v>9.0102000000000002E-2</v>
+        <v>0.14416399999999999</v>
       </c>
       <c r="AA13">
-        <v>9.5766000000000004E-2</v>
+        <v>0.153226</v>
       </c>
       <c r="AB13">
-        <v>9.4240000000000004E-2</v>
+        <v>0.150784</v>
       </c>
       <c r="AC13">
-        <v>9.9086999999999995E-2</v>
+        <v>0.15854499999999999</v>
       </c>
       <c r="AD13">
-        <v>0.106582</v>
+        <v>0.17053099999999999</v>
       </c>
       <c r="AE13">
-        <v>0.111766</v>
+        <v>0.17882600000000001</v>
       </c>
       <c r="AF13">
-        <v>9.8028000000000004E-2</v>
+        <v>0.15684500000000001</v>
       </c>
       <c r="AG13">
-        <v>0.104584</v>
+        <v>0.16733400000000001</v>
       </c>
       <c r="AH13">
-        <v>9.9945999999999993E-2</v>
+        <v>0.16089000000000001</v>
       </c>
       <c r="AI13">
-        <v>0.105529</v>
+        <v>0.168377</v>
       </c>
       <c r="AJ13">
-        <v>0.18155499999999999</v>
+        <v>0.29048800000000002</v>
       </c>
       <c r="AK13">
-        <v>0.17615800000000001</v>
+        <v>0.28185300000000002</v>
       </c>
       <c r="AL13">
-        <v>0.177013</v>
+        <v>0.28704400000000002</v>
       </c>
       <c r="AM13">
-        <v>0.17801700000000001</v>
+        <v>0.28708299999999998</v>
       </c>
       <c r="AN13">
-        <v>0.176763</v>
+        <v>0.28387800000000002</v>
       </c>
       <c r="AO13">
-        <v>0.18813199999999999</v>
+        <v>0.29844100000000001</v>
       </c>
       <c r="AP13">
         <v>53.582262</v>
@@ -9783,58 +9783,58 @@
         <v>29.377305</v>
       </c>
       <c r="X14">
-        <v>9.2424000000000006E-2</v>
+        <v>0.14787800000000001</v>
       </c>
       <c r="Y14">
-        <v>9.4077999999999995E-2</v>
+        <v>0.15027399999999999</v>
       </c>
       <c r="Z14">
-        <v>9.7742999999999997E-2</v>
+        <v>0.156389</v>
       </c>
       <c r="AA14">
-        <v>9.6556000000000003E-2</v>
+        <v>0.15448999999999999</v>
       </c>
       <c r="AB14">
-        <v>9.5426999999999998E-2</v>
+        <v>0.15268300000000001</v>
       </c>
       <c r="AC14">
-        <v>0.110233</v>
+        <v>0.17639299999999999</v>
       </c>
       <c r="AD14">
-        <v>0.104924</v>
+        <v>0.167879</v>
       </c>
       <c r="AE14">
-        <v>0.110404</v>
+        <v>0.176646</v>
       </c>
       <c r="AF14">
-        <v>0.103877</v>
+        <v>0.16620399999999999</v>
       </c>
       <c r="AG14">
-        <v>0.108545</v>
+        <v>0.17367199999999999</v>
       </c>
       <c r="AH14">
-        <v>9.8016000000000006E-2</v>
+        <v>0.15813099999999999</v>
       </c>
       <c r="AI14">
-        <v>0.102515</v>
+        <v>0.16377800000000001</v>
       </c>
       <c r="AJ14">
-        <v>0.182334</v>
+        <v>0.29173500000000002</v>
       </c>
       <c r="AK14">
-        <v>0.17569799999999999</v>
+        <v>0.28111700000000001</v>
       </c>
       <c r="AL14">
-        <v>0.183196</v>
+        <v>0.29323100000000002</v>
       </c>
       <c r="AM14">
-        <v>0.17780199999999999</v>
+        <v>0.285991</v>
       </c>
       <c r="AN14">
-        <v>0.176596</v>
+        <v>0.282001</v>
       </c>
       <c r="AO14">
-        <v>0.18615000000000001</v>
+        <v>0.29603099999999999</v>
       </c>
       <c r="AP14">
         <v>52.775505000000003</v>
@@ -9995,58 +9995,58 @@
         <v>28.252735999999999</v>
       </c>
       <c r="X15">
-        <v>9.1470999999999997E-2</v>
+        <v>0.14635300000000001</v>
       </c>
       <c r="Y15">
-        <v>9.0979000000000004E-2</v>
+        <v>0.14666799999999999</v>
       </c>
       <c r="Z15">
-        <v>9.5296000000000006E-2</v>
+        <v>0.152473</v>
       </c>
       <c r="AA15">
-        <v>8.6121000000000003E-2</v>
+        <v>0.137794</v>
       </c>
       <c r="AB15">
-        <v>8.7182999999999997E-2</v>
+        <v>0.13949400000000001</v>
       </c>
       <c r="AC15">
-        <v>8.3797999999999997E-2</v>
+        <v>0.134071</v>
       </c>
       <c r="AD15">
-        <v>0.103764</v>
+        <v>0.166022</v>
       </c>
       <c r="AE15">
-        <v>0.10703600000000001</v>
+        <v>0.17125699999999999</v>
       </c>
       <c r="AF15">
-        <v>0.102649</v>
+        <v>0.164238</v>
       </c>
       <c r="AG15">
-        <v>0.103172</v>
+        <v>0.165074</v>
       </c>
       <c r="AH15">
-        <v>9.3925999999999996E-2</v>
+        <v>0.15251899999999999</v>
       </c>
       <c r="AI15">
-        <v>9.5835000000000004E-2</v>
+        <v>0.15428600000000001</v>
       </c>
       <c r="AJ15">
-        <v>0.17943400000000001</v>
+        <v>0.28709499999999999</v>
       </c>
       <c r="AK15">
-        <v>0.17054</v>
+        <v>0.272864</v>
       </c>
       <c r="AL15">
-        <v>0.18234500000000001</v>
+        <v>0.29315400000000003</v>
       </c>
       <c r="AM15">
-        <v>0.171959</v>
+        <v>0.28021200000000002</v>
       </c>
       <c r="AN15">
-        <v>0.17052800000000001</v>
+        <v>0.27552300000000002</v>
       </c>
       <c r="AO15">
-        <v>0.18044399999999999</v>
+        <v>0.29056100000000001</v>
       </c>
       <c r="AP15">
         <v>52.9206</v>
@@ -10207,58 +10207,58 @@
         <v>27.815975999999999</v>
       </c>
       <c r="X16">
-        <v>9.0887999999999997E-2</v>
+        <v>0.14541999999999999</v>
       </c>
       <c r="Y16">
-        <v>9.1655E-2</v>
+        <v>0.145317</v>
       </c>
       <c r="Z16">
-        <v>9.2704999999999996E-2</v>
+        <v>0.14832899999999999</v>
       </c>
       <c r="AA16">
-        <v>9.1904E-2</v>
+        <v>0.14704600000000001</v>
       </c>
       <c r="AB16">
-        <v>9.0739E-2</v>
+        <v>0.14518200000000001</v>
       </c>
       <c r="AC16">
-        <v>8.4690000000000001E-2</v>
+        <v>0.13550000000000001</v>
       </c>
       <c r="AD16">
-        <v>0.10302699999999999</v>
+        <v>0.16484299999999999</v>
       </c>
       <c r="AE16">
-        <v>0.103612</v>
+        <v>0.16578000000000001</v>
       </c>
       <c r="AF16">
-        <v>0.10674400000000001</v>
+        <v>0.17079</v>
       </c>
       <c r="AG16">
-        <v>0.105114</v>
+        <v>0.168183</v>
       </c>
       <c r="AH16">
-        <v>9.3905000000000002E-2</v>
+        <v>0.15255199999999999</v>
       </c>
       <c r="AI16">
-        <v>9.5389000000000002E-2</v>
+        <v>0.153419</v>
       </c>
       <c r="AJ16">
-        <v>0.17683699999999999</v>
+        <v>0.282939</v>
       </c>
       <c r="AK16">
-        <v>0.165687</v>
+        <v>0.2651</v>
       </c>
       <c r="AL16">
-        <v>0.18865100000000001</v>
+        <v>0.30029499999999998</v>
       </c>
       <c r="AM16">
-        <v>0.17700299999999999</v>
+        <v>0.28522199999999998</v>
       </c>
       <c r="AN16">
-        <v>0.170042</v>
+        <v>0.27368399999999998</v>
       </c>
       <c r="AO16">
-        <v>0.180196</v>
+        <v>0.28967199999999999</v>
       </c>
       <c r="AP16">
         <v>54.059849</v>
@@ -10419,58 +10419,58 @@
         <v>28.072616</v>
       </c>
       <c r="X17">
-        <v>8.8305999999999996E-2</v>
+        <v>0.14129</v>
       </c>
       <c r="Y17">
-        <v>8.3612000000000006E-2</v>
+        <v>0.13791500000000001</v>
       </c>
       <c r="Z17">
-        <v>8.8030999999999998E-2</v>
+        <v>0.140849</v>
       </c>
       <c r="AA17">
-        <v>8.8253999999999999E-2</v>
+        <v>0.141206</v>
       </c>
       <c r="AB17">
-        <v>8.7232000000000004E-2</v>
+        <v>0.139572</v>
       </c>
       <c r="AC17">
-        <v>8.6915999999999993E-2</v>
+        <v>0.13906399999999999</v>
       </c>
       <c r="AD17">
-        <v>0.10352500000000001</v>
+        <v>0.16564000000000001</v>
       </c>
       <c r="AE17">
-        <v>9.7978999999999997E-2</v>
+        <v>0.15676699999999999</v>
       </c>
       <c r="AF17">
-        <v>0.10381</v>
+        <v>0.16609599999999999</v>
       </c>
       <c r="AG17">
-        <v>9.7835000000000005E-2</v>
+        <v>0.15653700000000001</v>
       </c>
       <c r="AH17">
-        <v>9.2438000000000006E-2</v>
+        <v>0.15080199999999999</v>
       </c>
       <c r="AI17">
-        <v>9.7424999999999998E-2</v>
+        <v>0.15614</v>
       </c>
       <c r="AJ17">
-        <v>0.173041</v>
+        <v>0.276866</v>
       </c>
       <c r="AK17">
-        <v>0.15875300000000001</v>
+        <v>0.25400400000000001</v>
       </c>
       <c r="AL17">
-        <v>0.184812</v>
+        <v>0.29652000000000001</v>
       </c>
       <c r="AM17">
-        <v>0.168132</v>
+        <v>0.27583299999999999</v>
       </c>
       <c r="AN17">
-        <v>0.164795</v>
+        <v>0.26858799999999999</v>
       </c>
       <c r="AO17">
-        <v>0.18056900000000001</v>
+        <v>0.28954800000000003</v>
       </c>
       <c r="AP17">
         <v>55.167695000000002</v>

</xml_diff>